<commit_message>
Estadisticos Segundo Parcial 20241 Rescatables 4
</commit_message>
<xml_diff>
--- a/docentes/Avila Coronado Julieta - Estadisticos 20241.xlsx
+++ b/docentes/Avila Coronado Julieta - Estadisticos 20241.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="39">
   <si>
     <t>Mat</t>
   </si>
@@ -82,6 +82,12 @@
     <t>Reprobadas</t>
   </si>
   <si>
+    <t>TELLO</t>
+  </si>
+  <si>
+    <t>MONTERD</t>
+  </si>
+  <si>
     <t>LUNA</t>
   </si>
   <si>
@@ -94,6 +100,12 @@
     <t>MONTIEL</t>
   </si>
   <si>
+    <t>DE LA LUZ</t>
+  </si>
+  <si>
+    <t>VENTURA</t>
+  </si>
+  <si>
     <t>SANCHEZ</t>
   </si>
   <si>
@@ -104,6 +116,12 @@
   </si>
   <si>
     <t>CONTRERAS</t>
+  </si>
+  <si>
+    <t>EMMANUEL</t>
+  </si>
+  <si>
+    <t>ANGEL YAMIL</t>
   </si>
   <si>
     <t>JUAN YAHEL</t>
@@ -1058,7 +1076,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="15.7109375" customWidth="1"/>
@@ -1090,16 +1108,16 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
-        <v>23330051920015</v>
+        <v>23330051920022</v>
       </c>
       <c r="B2" t="s">
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -1108,50 +1126,50 @@
         <v>9</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
-        <v>23330051920263</v>
+        <v>23330051920017</v>
       </c>
       <c r="B3" t="s">
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
-        <v>23330051920045</v>
+        <v>23330051920015</v>
       </c>
       <c r="B4" t="s">
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G4">
         <v>2</v>
@@ -1159,16 +1177,16 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5">
-        <v>23330051920259</v>
+        <v>23330051920263</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
         <v>8</v>
@@ -1177,6 +1195,52 @@
         <v>12</v>
       </c>
       <c r="G5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>23330051920045</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>23330051920259</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7">
         <v>1</v>
       </c>
     </row>

</xml_diff>